<commit_message>
feat: 新增 set_desktop_layout 桌面布局设置方法、桌面设置新增 set_desktop_setting 开关方法 query_desktop_setting(item) - param:item - 查询桌面设置项状态 set_desktop_setting(item, desired) - param: item, 'on'/'off' - 开关桌面设置项（） set_desktop_layout(layout_name)	- param:'标准' / '紧凑' - 设置桌面布局
</commit_message>
<xml_diff>
--- a/HarmonyOS_API汇总.xlsx
+++ b/HarmonyOS_API汇总.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R17"/>
+  <dimension ref="A1:T17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -478,6 +478,8 @@
     <col width="30" customWidth="1" min="16" max="16"/>
     <col width="30" customWidth="1" min="17" max="17"/>
     <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
+    <col width="30" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -525,16 +527,22 @@
       <c r="N1" s="2" t="n"/>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>电池</t>
+          <t>桌面设置</t>
         </is>
       </c>
       <c r="P1" s="2" t="n"/>
       <c r="Q1" s="1" t="inlineStr">
         <is>
+          <t>电池</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="n"/>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>通知与免打扰</t>
         </is>
       </c>
-      <c r="R1" s="2" t="n"/>
+      <c r="T1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -623,6 +631,16 @@
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>设置项</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>API</t>
         </is>
@@ -707,21 +725,34 @@
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
+          <t>桌面设置(下滑/上滑/布局/自动对齐/锁定布局)</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="inlineStr">
+        <is>
+          <t>query_desktop_setting(item)
+set_desktop_setting(item, 'on'/'off')
+set_desktop_layout('标准'/'紧凑')
+  item: swipe_down/swipe_up/layout/auto_align/lock_layout</t>
+        </is>
+      </c>
+      <c r="Q3" s="4" t="inlineStr">
+        <is>
           <t>省电模式</t>
         </is>
       </c>
-      <c r="P3" s="4" t="inlineStr">
+      <c r="R3" s="4" t="inlineStr">
         <is>
           <t>query_power_saving()
 set_power_saving('on'/'off')</t>
         </is>
       </c>
-      <c r="Q3" s="4" t="inlineStr">
+      <c r="S3" s="4" t="inlineStr">
         <is>
           <t>勿扰模式</t>
         </is>
       </c>
-      <c r="R3" s="4" t="inlineStr">
+      <c r="T3" s="4" t="inlineStr">
         <is>
           <t>query_dnd()
 set_dnd('on'/'off')</t>
@@ -809,6 +840,8 @@
       <c r="P4" s="5" t="inlineStr"/>
       <c r="Q4" s="5" t="inlineStr"/>
       <c r="R4" s="5" t="inlineStr"/>
+      <c r="S4" s="5" t="inlineStr"/>
+      <c r="T4" s="5" t="inlineStr"/>
     </row>
     <row r="5" ht="50" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -881,6 +914,8 @@
       <c r="P5" s="5" t="inlineStr"/>
       <c r="Q5" s="5" t="inlineStr"/>
       <c r="R5" s="5" t="inlineStr"/>
+      <c r="S5" s="5" t="inlineStr"/>
+      <c r="T5" s="5" t="inlineStr"/>
     </row>
     <row r="6" ht="50" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -955,6 +990,8 @@
       <c r="P6" s="5" t="inlineStr"/>
       <c r="Q6" s="5" t="inlineStr"/>
       <c r="R6" s="5" t="inlineStr"/>
+      <c r="S6" s="5" t="inlineStr"/>
+      <c r="T6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="50" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -1018,6 +1055,8 @@
       <c r="P7" s="5" t="inlineStr"/>
       <c r="Q7" s="5" t="inlineStr"/>
       <c r="R7" s="5" t="inlineStr"/>
+      <c r="S7" s="5" t="inlineStr"/>
+      <c r="T7" s="5" t="inlineStr"/>
     </row>
     <row r="8" ht="50" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -1056,6 +1095,8 @@
       <c r="P8" s="5" t="inlineStr"/>
       <c r="Q8" s="5" t="inlineStr"/>
       <c r="R8" s="5" t="inlineStr"/>
+      <c r="S8" s="5" t="inlineStr"/>
+      <c r="T8" s="5" t="inlineStr"/>
     </row>
     <row r="9" ht="50" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -1093,6 +1134,8 @@
       <c r="P9" s="5" t="inlineStr"/>
       <c r="Q9" s="5" t="inlineStr"/>
       <c r="R9" s="5" t="inlineStr"/>
+      <c r="S9" s="5" t="inlineStr"/>
+      <c r="T9" s="5" t="inlineStr"/>
     </row>
     <row r="10" ht="50" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
@@ -1131,6 +1174,8 @@
       <c r="P10" s="5" t="inlineStr"/>
       <c r="Q10" s="5" t="inlineStr"/>
       <c r="R10" s="5" t="inlineStr"/>
+      <c r="S10" s="5" t="inlineStr"/>
+      <c r="T10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="50" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -1169,6 +1214,8 @@
       <c r="P11" s="5" t="inlineStr"/>
       <c r="Q11" s="5" t="inlineStr"/>
       <c r="R11" s="5" t="inlineStr"/>
+      <c r="S11" s="5" t="inlineStr"/>
+      <c r="T11" s="5" t="inlineStr"/>
     </row>
     <row r="12" ht="50" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -1206,6 +1253,8 @@
       <c r="P12" s="5" t="inlineStr"/>
       <c r="Q12" s="5" t="inlineStr"/>
       <c r="R12" s="5" t="inlineStr"/>
+      <c r="S12" s="5" t="inlineStr"/>
+      <c r="T12" s="5" t="inlineStr"/>
     </row>
     <row r="13" ht="50" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -1243,6 +1292,8 @@
       <c r="P13" s="5" t="inlineStr"/>
       <c r="Q13" s="5" t="inlineStr"/>
       <c r="R13" s="5" t="inlineStr"/>
+      <c r="S13" s="5" t="inlineStr"/>
+      <c r="T13" s="5" t="inlineStr"/>
     </row>
     <row r="14" ht="50" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
@@ -1272,6 +1323,8 @@
       <c r="P14" s="5" t="inlineStr"/>
       <c r="Q14" s="5" t="inlineStr"/>
       <c r="R14" s="5" t="inlineStr"/>
+      <c r="S14" s="5" t="inlineStr"/>
+      <c r="T14" s="5" t="inlineStr"/>
     </row>
     <row r="15" ht="50" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -1301,6 +1354,8 @@
       <c r="P15" s="5" t="inlineStr"/>
       <c r="Q15" s="5" t="inlineStr"/>
       <c r="R15" s="5" t="inlineStr"/>
+      <c r="S15" s="5" t="inlineStr"/>
+      <c r="T15" s="5" t="inlineStr"/>
     </row>
     <row r="16" ht="50" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
@@ -1330,6 +1385,8 @@
       <c r="P16" s="5" t="inlineStr"/>
       <c r="Q16" s="5" t="inlineStr"/>
       <c r="R16" s="5" t="inlineStr"/>
+      <c r="S16" s="5" t="inlineStr"/>
+      <c r="T16" s="5" t="inlineStr"/>
     </row>
     <row r="17" ht="50" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -1359,14 +1416,17 @@
       <c r="P17" s="5" t="inlineStr"/>
       <c r="Q17" s="5" t="inlineStr"/>
       <c r="R17" s="5" t="inlineStr"/>
+      <c r="S17" s="5" t="inlineStr"/>
+      <c r="T17" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="Q1:R1"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="K1:L1"/>
+    <mergeCell ref="S1:T1"/>
     <mergeCell ref="O1:P1"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="M1:N1"/>

</xml_diff>